<commit_message>
Versão 1.0.6: assinatura e logo no cabeçalho e nas planilhas RDO/FT.
Adiciona gestão de assinatura e logo na aba Cabeçalhos, inserção proporcional no Excel, data de geração no RDO, modelo de cabeçalho com imagens em template/, e Pillow no .exe; actualiza manual e README.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/template/RDO.xlsx
+++ b/template/RDO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorio\Gerar_Relatorio\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EA3844-0D31-41F1-95F8-6C79A23E6F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7A7D9B-74C5-4637-BCCF-8FCBC2016371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-6550" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" 2026-01-01" sheetId="2" r:id="rId1"/>
@@ -881,13 +881,13 @@
     <t>VISTO:</t>
   </si>
   <si>
-    <t>________________________</t>
+    <t xml:space="preserve">EMPREENDIMENTO:  </t>
   </si>
   <si>
-    <t>_____________________</t>
+    <t>______________________________</t>
   </si>
   <si>
-    <t xml:space="preserve">EMPREENDIMENTO:  </t>
+    <t>_________________________</t>
   </si>
 </sst>
 </file>
@@ -2054,128 +2054,125 @@
     <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="23" fillId="0" borderId="59" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="23" fillId="0" borderId="60" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="23" fillId="0" borderId="61" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="24" fillId="0" borderId="59" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="24" fillId="0" borderId="60" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="24" fillId="0" borderId="61" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="66" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="67" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="18" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="18" fillId="0" borderId="64" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="66" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="67" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
@@ -2186,6 +2183,33 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="47" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="52" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="57" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="47" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2204,151 +2228,127 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="47" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="52" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="57" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="56" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="64" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="66" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="67" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="18" fillId="0" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="18" fillId="0" borderId="64" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="66" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="67" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="23" fillId="0" borderId="59" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="23" fillId="0" borderId="60" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="23" fillId="0" borderId="61" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="24" fillId="0" borderId="59" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="24" fillId="0" borderId="60" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="24" fillId="0" borderId="61" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7742,56 +7742,56 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="5"/>
-      <c r="H1" s="56" t="s">
+      <c r="H1" s="134" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="58"/>
-      <c r="J1" s="60" t="s">
+      <c r="I1" s="136"/>
+      <c r="J1" s="138" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="62"/>
+      <c r="K1" s="140"/>
     </row>
     <row r="2" spans="2:11" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="7"/>
       <c r="C2" s="8"/>
-      <c r="D2" s="64" t="s">
+      <c r="D2" s="142" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="63"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="135"/>
+      <c r="I2" s="137"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="141"/>
     </row>
     <row r="3" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="7"/>
       <c r="C3" s="8"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="66" t="s">
+      <c r="D3" s="143"/>
+      <c r="E3" s="143"/>
+      <c r="F3" s="143"/>
+      <c r="G3" s="143"/>
+      <c r="H3" s="144" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="67"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="63"/>
+      <c r="I3" s="145"/>
+      <c r="J3" s="139"/>
+      <c r="K3" s="141"/>
     </row>
     <row r="4" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="7"/>
       <c r="C4" s="8"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="67"/>
-      <c r="J4" s="66" t="s">
+      <c r="D4" s="143"/>
+      <c r="E4" s="143"/>
+      <c r="F4" s="143"/>
+      <c r="G4" s="143"/>
+      <c r="H4" s="144"/>
+      <c r="I4" s="145"/>
+      <c r="J4" s="144" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="69"/>
+      <c r="K4" s="147"/>
     </row>
     <row r="5" spans="2:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="7"/>
@@ -7804,34 +7804,34 @@
         <v>5</v>
       </c>
       <c r="I5" s="14"/>
-      <c r="J5" s="68"/>
-      <c r="K5" s="70"/>
+      <c r="J5" s="146"/>
+      <c r="K5" s="148"/>
     </row>
     <row r="6" spans="2:11" ht="14.45" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B6" s="7"/>
-      <c r="C6" s="50" t="s">
-        <v>32</v>
+      <c r="C6" s="128" t="s">
+        <v>30</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="53"/>
+      <c r="D6" s="130"/>
+      <c r="E6" s="130"/>
+      <c r="F6" s="130"/>
+      <c r="G6" s="130"/>
+      <c r="H6" s="130"/>
+      <c r="I6" s="130"/>
+      <c r="J6" s="130"/>
+      <c r="K6" s="131"/>
     </row>
     <row r="7" spans="2:11" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
-      <c r="I7" s="54"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="55"/>
+      <c r="C7" s="129"/>
+      <c r="D7" s="132"/>
+      <c r="E7" s="132"/>
+      <c r="F7" s="132"/>
+      <c r="G7" s="132"/>
+      <c r="H7" s="132"/>
+      <c r="I7" s="132"/>
+      <c r="J7" s="132"/>
+      <c r="K7" s="133"/>
     </row>
     <row r="8" spans="2:11" ht="12.75" x14ac:dyDescent="0.25">
       <c r="B8" s="7"/>
@@ -7839,27 +7839,27 @@
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="17"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="72"/>
-      <c r="I8" s="72"/>
-      <c r="J8" s="72"/>
-      <c r="K8" s="73"/>
+      <c r="G8" s="120"/>
+      <c r="H8" s="121"/>
+      <c r="I8" s="121"/>
+      <c r="J8" s="121"/>
+      <c r="K8" s="122"/>
     </row>
     <row r="9" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="7"/>
       <c r="C9" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="75"/>
-      <c r="G9" s="76" t="s">
+      <c r="D9" s="123"/>
+      <c r="E9" s="123"/>
+      <c r="F9" s="124"/>
+      <c r="G9" s="125" t="s">
         <v>7</v>
       </c>
-      <c r="H9" s="77"/>
-      <c r="I9" s="77"/>
-      <c r="J9" s="77"/>
-      <c r="K9" s="78"/>
+      <c r="H9" s="126"/>
+      <c r="I9" s="126"/>
+      <c r="J9" s="126"/>
+      <c r="K9" s="127"/>
     </row>
     <row r="10" spans="2:11" ht="12.75" x14ac:dyDescent="0.25">
       <c r="B10" s="7"/>
@@ -7867,11 +7867,11 @@
       <c r="D10" s="20"/>
       <c r="E10" s="20"/>
       <c r="F10" s="21"/>
-      <c r="G10" s="79"/>
-      <c r="H10" s="80"/>
-      <c r="I10" s="80"/>
-      <c r="J10" s="80"/>
-      <c r="K10" s="81"/>
+      <c r="G10" s="108"/>
+      <c r="H10" s="109"/>
+      <c r="I10" s="109"/>
+      <c r="J10" s="109"/>
+      <c r="K10" s="110"/>
     </row>
     <row r="11" spans="2:11" ht="12.75" x14ac:dyDescent="0.25">
       <c r="B11" s="7"/>
@@ -7881,11 +7881,11 @@
       <c r="D11" s="23"/>
       <c r="E11" s="24"/>
       <c r="F11" s="25"/>
-      <c r="G11" s="79"/>
-      <c r="H11" s="80"/>
-      <c r="I11" s="80"/>
-      <c r="J11" s="80"/>
-      <c r="K11" s="81"/>
+      <c r="G11" s="108"/>
+      <c r="H11" s="109"/>
+      <c r="I11" s="109"/>
+      <c r="J11" s="109"/>
+      <c r="K11" s="110"/>
     </row>
     <row r="12" spans="2:11" ht="12.75" x14ac:dyDescent="0.25">
       <c r="B12" s="7"/>
@@ -7893,11 +7893,11 @@
       <c r="D12" s="20"/>
       <c r="E12" s="26"/>
       <c r="F12" s="21"/>
-      <c r="G12" s="79"/>
-      <c r="H12" s="80"/>
-      <c r="I12" s="80"/>
-      <c r="J12" s="80"/>
-      <c r="K12" s="81"/>
+      <c r="G12" s="108"/>
+      <c r="H12" s="109"/>
+      <c r="I12" s="109"/>
+      <c r="J12" s="109"/>
+      <c r="K12" s="110"/>
     </row>
     <row r="13" spans="2:11" ht="12.75" x14ac:dyDescent="0.25">
       <c r="B13" s="7"/>
@@ -7907,11 +7907,11 @@
       <c r="D13" s="23"/>
       <c r="E13" s="24"/>
       <c r="F13" s="25"/>
-      <c r="G13" s="79"/>
-      <c r="H13" s="80"/>
-      <c r="I13" s="80"/>
-      <c r="J13" s="80"/>
-      <c r="K13" s="81"/>
+      <c r="G13" s="108"/>
+      <c r="H13" s="109"/>
+      <c r="I13" s="109"/>
+      <c r="J13" s="109"/>
+      <c r="K13" s="110"/>
     </row>
     <row r="14" spans="2:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="7"/>
@@ -7919,748 +7919,748 @@
       <c r="D14" s="28"/>
       <c r="E14" s="29"/>
       <c r="F14" s="30"/>
-      <c r="G14" s="82"/>
-      <c r="H14" s="83"/>
-      <c r="I14" s="83"/>
-      <c r="J14" s="83"/>
-      <c r="K14" s="84"/>
+      <c r="G14" s="111"/>
+      <c r="H14" s="112"/>
+      <c r="I14" s="112"/>
+      <c r="J14" s="112"/>
+      <c r="K14" s="113"/>
     </row>
     <row r="15" spans="2:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="7"/>
-      <c r="C15" s="85" t="s">
+      <c r="C15" s="114" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="86"/>
-      <c r="E15" s="86"/>
-      <c r="F15" s="87"/>
+      <c r="D15" s="115"/>
+      <c r="E15" s="115"/>
+      <c r="F15" s="116"/>
       <c r="G15" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="H15" s="88" t="s">
+      <c r="H15" s="117" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="89"/>
-      <c r="J15" s="89"/>
-      <c r="K15" s="90"/>
+      <c r="I15" s="118"/>
+      <c r="J15" s="118"/>
+      <c r="K15" s="119"/>
     </row>
     <row r="16" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="91" t="s">
+      <c r="B16" s="90" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="106"/>
-      <c r="D16" s="107"/>
-      <c r="E16" s="107"/>
-      <c r="F16" s="108"/>
-      <c r="G16" s="94"/>
-      <c r="H16" s="97"/>
-      <c r="I16" s="98"/>
-      <c r="J16" s="98"/>
-      <c r="K16" s="99"/>
+      <c r="C16" s="84"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="85"/>
+      <c r="F16" s="86"/>
+      <c r="G16" s="102"/>
+      <c r="H16" s="105"/>
+      <c r="I16" s="106"/>
+      <c r="J16" s="106"/>
+      <c r="K16" s="107"/>
     </row>
     <row r="17" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="92"/>
-      <c r="C17" s="109"/>
-      <c r="D17" s="110"/>
-      <c r="E17" s="110"/>
-      <c r="F17" s="111"/>
-      <c r="G17" s="95"/>
-      <c r="H17" s="100"/>
-      <c r="I17" s="101"/>
-      <c r="J17" s="101"/>
-      <c r="K17" s="102"/>
+      <c r="B17" s="91"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="88"/>
+      <c r="E17" s="88"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="103"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="52"/>
     </row>
     <row r="18" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="92"/>
-      <c r="C18" s="109"/>
-      <c r="D18" s="110"/>
-      <c r="E18" s="110"/>
-      <c r="F18" s="111"/>
-      <c r="G18" s="95"/>
-      <c r="H18" s="100"/>
-      <c r="I18" s="101"/>
-      <c r="J18" s="101"/>
-      <c r="K18" s="102"/>
+      <c r="B18" s="91"/>
+      <c r="C18" s="87"/>
+      <c r="D18" s="88"/>
+      <c r="E18" s="88"/>
+      <c r="F18" s="89"/>
+      <c r="G18" s="103"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="51"/>
+      <c r="K18" s="52"/>
       <c r="L18" s="32"/>
     </row>
     <row r="19" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="92"/>
-      <c r="C19" s="109"/>
-      <c r="D19" s="110"/>
-      <c r="E19" s="110"/>
-      <c r="F19" s="111"/>
-      <c r="G19" s="95"/>
-      <c r="H19" s="100"/>
-      <c r="I19" s="101"/>
-      <c r="J19" s="101"/>
-      <c r="K19" s="102"/>
+      <c r="B19" s="91"/>
+      <c r="C19" s="87"/>
+      <c r="D19" s="88"/>
+      <c r="E19" s="88"/>
+      <c r="F19" s="89"/>
+      <c r="G19" s="103"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="52"/>
       <c r="L19" s="33"/>
     </row>
     <row r="20" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="92"/>
-      <c r="C20" s="109"/>
-      <c r="D20" s="110"/>
-      <c r="E20" s="110"/>
-      <c r="F20" s="111"/>
-      <c r="G20" s="95"/>
-      <c r="H20" s="100"/>
-      <c r="I20" s="101"/>
-      <c r="J20" s="101"/>
-      <c r="K20" s="102"/>
+      <c r="B20" s="91"/>
+      <c r="C20" s="87"/>
+      <c r="D20" s="88"/>
+      <c r="E20" s="88"/>
+      <c r="F20" s="89"/>
+      <c r="G20" s="103"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="51"/>
+      <c r="K20" s="52"/>
       <c r="L20" s="33"/>
     </row>
     <row r="21" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="92"/>
-      <c r="C21" s="109"/>
-      <c r="D21" s="110"/>
-      <c r="E21" s="110"/>
-      <c r="F21" s="111"/>
-      <c r="G21" s="95"/>
-      <c r="H21" s="100"/>
-      <c r="I21" s="101"/>
-      <c r="J21" s="101"/>
-      <c r="K21" s="102"/>
+      <c r="B21" s="91"/>
+      <c r="C21" s="87"/>
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="F21" s="89"/>
+      <c r="G21" s="103"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="51"/>
+      <c r="K21" s="52"/>
       <c r="L21" s="33"/>
     </row>
     <row r="22" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="92"/>
-      <c r="C22" s="109"/>
-      <c r="D22" s="110"/>
-      <c r="E22" s="110"/>
-      <c r="F22" s="111"/>
-      <c r="G22" s="95"/>
-      <c r="H22" s="100"/>
-      <c r="I22" s="101"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="102"/>
+      <c r="B22" s="91"/>
+      <c r="C22" s="87"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="88"/>
+      <c r="F22" s="89"/>
+      <c r="G22" s="103"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="51"/>
+      <c r="K22" s="52"/>
       <c r="L22" s="33"/>
     </row>
     <row r="23" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="92"/>
-      <c r="C23" s="109"/>
-      <c r="D23" s="110"/>
-      <c r="E23" s="110"/>
-      <c r="F23" s="111"/>
-      <c r="G23" s="95"/>
-      <c r="H23" s="100"/>
-      <c r="I23" s="101"/>
-      <c r="J23" s="101"/>
-      <c r="K23" s="102"/>
+      <c r="B23" s="91"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="88"/>
+      <c r="F23" s="89"/>
+      <c r="G23" s="103"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="51"/>
+      <c r="K23" s="52"/>
       <c r="L23" s="33"/>
     </row>
     <row r="24" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="92"/>
-      <c r="C24" s="109"/>
-      <c r="D24" s="110"/>
-      <c r="E24" s="110"/>
-      <c r="F24" s="111"/>
-      <c r="G24" s="95"/>
-      <c r="H24" s="100"/>
-      <c r="I24" s="101"/>
-      <c r="J24" s="101"/>
-      <c r="K24" s="102"/>
+      <c r="B24" s="91"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="89"/>
+      <c r="G24" s="103"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="52"/>
       <c r="L24" s="33"/>
     </row>
     <row r="25" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="92"/>
-      <c r="C25" s="109"/>
-      <c r="D25" s="110"/>
-      <c r="E25" s="110"/>
-      <c r="F25" s="111"/>
-      <c r="G25" s="95"/>
-      <c r="H25" s="100"/>
-      <c r="I25" s="101"/>
-      <c r="J25" s="101"/>
-      <c r="K25" s="102"/>
+      <c r="B25" s="91"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="88"/>
+      <c r="E25" s="88"/>
+      <c r="F25" s="89"/>
+      <c r="G25" s="103"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="51"/>
+      <c r="K25" s="52"/>
       <c r="L25" s="33"/>
     </row>
     <row r="26" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="92"/>
-      <c r="C26" s="109"/>
-      <c r="D26" s="110"/>
-      <c r="E26" s="110"/>
-      <c r="F26" s="111"/>
-      <c r="G26" s="95"/>
-      <c r="H26" s="100"/>
-      <c r="I26" s="101"/>
-      <c r="J26" s="101"/>
-      <c r="K26" s="102"/>
+      <c r="B26" s="91"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="88"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="89"/>
+      <c r="G26" s="103"/>
+      <c r="H26" s="50"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="52"/>
       <c r="L26" s="32"/>
     </row>
     <row r="27" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="92"/>
-      <c r="C27" s="109"/>
-      <c r="D27" s="110"/>
-      <c r="E27" s="110"/>
-      <c r="F27" s="111"/>
-      <c r="G27" s="95"/>
-      <c r="H27" s="100"/>
-      <c r="I27" s="101"/>
-      <c r="J27" s="101"/>
-      <c r="K27" s="102"/>
+      <c r="B27" s="91"/>
+      <c r="C27" s="87"/>
+      <c r="D27" s="88"/>
+      <c r="E27" s="88"/>
+      <c r="F27" s="89"/>
+      <c r="G27" s="103"/>
+      <c r="H27" s="50"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="52"/>
       <c r="L27" s="32"/>
     </row>
     <row r="28" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="92"/>
-      <c r="C28" s="109"/>
-      <c r="D28" s="110"/>
-      <c r="E28" s="110"/>
-      <c r="F28" s="111"/>
-      <c r="G28" s="95"/>
-      <c r="H28" s="100"/>
-      <c r="I28" s="101"/>
-      <c r="J28" s="101"/>
-      <c r="K28" s="102"/>
+      <c r="B28" s="91"/>
+      <c r="C28" s="87"/>
+      <c r="D28" s="88"/>
+      <c r="E28" s="88"/>
+      <c r="F28" s="89"/>
+      <c r="G28" s="103"/>
+      <c r="H28" s="50"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="51"/>
+      <c r="K28" s="52"/>
       <c r="L28" s="33"/>
     </row>
     <row r="29" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="92"/>
-      <c r="C29" s="109"/>
-      <c r="D29" s="110"/>
-      <c r="E29" s="110"/>
-      <c r="F29" s="111"/>
-      <c r="G29" s="95"/>
-      <c r="H29" s="100"/>
-      <c r="I29" s="101"/>
-      <c r="J29" s="101"/>
-      <c r="K29" s="102"/>
+      <c r="B29" s="91"/>
+      <c r="C29" s="87"/>
+      <c r="D29" s="88"/>
+      <c r="E29" s="88"/>
+      <c r="F29" s="89"/>
+      <c r="G29" s="103"/>
+      <c r="H29" s="50"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="52"/>
       <c r="L29" s="32"/>
     </row>
     <row r="30" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="92"/>
-      <c r="C30" s="109"/>
-      <c r="D30" s="110"/>
-      <c r="E30" s="110"/>
-      <c r="F30" s="111"/>
-      <c r="G30" s="95"/>
-      <c r="H30" s="100"/>
-      <c r="I30" s="101"/>
-      <c r="J30" s="101"/>
-      <c r="K30" s="102"/>
+      <c r="B30" s="91"/>
+      <c r="C30" s="87"/>
+      <c r="D30" s="88"/>
+      <c r="E30" s="88"/>
+      <c r="F30" s="89"/>
+      <c r="G30" s="103"/>
+      <c r="H30" s="50"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="51"/>
+      <c r="K30" s="52"/>
       <c r="L30" s="32"/>
     </row>
     <row r="31" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="92"/>
-      <c r="C31" s="109"/>
-      <c r="D31" s="110"/>
-      <c r="E31" s="110"/>
-      <c r="F31" s="111"/>
-      <c r="G31" s="95"/>
-      <c r="H31" s="100"/>
-      <c r="I31" s="101"/>
-      <c r="J31" s="101"/>
-      <c r="K31" s="102"/>
+      <c r="B31" s="91"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="88"/>
+      <c r="E31" s="88"/>
+      <c r="F31" s="89"/>
+      <c r="G31" s="103"/>
+      <c r="H31" s="50"/>
+      <c r="I31" s="51"/>
+      <c r="J31" s="51"/>
+      <c r="K31" s="52"/>
       <c r="L31" s="32"/>
     </row>
     <row r="32" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="92"/>
-      <c r="C32" s="109"/>
-      <c r="D32" s="110"/>
-      <c r="E32" s="110"/>
-      <c r="F32" s="111"/>
-      <c r="G32" s="95"/>
-      <c r="H32" s="100"/>
-      <c r="I32" s="101"/>
-      <c r="J32" s="101"/>
-      <c r="K32" s="102"/>
+      <c r="B32" s="91"/>
+      <c r="C32" s="87"/>
+      <c r="D32" s="88"/>
+      <c r="E32" s="88"/>
+      <c r="F32" s="89"/>
+      <c r="G32" s="103"/>
+      <c r="H32" s="50"/>
+      <c r="I32" s="51"/>
+      <c r="J32" s="51"/>
+      <c r="K32" s="52"/>
       <c r="L32" s="32"/>
     </row>
     <row r="33" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="92"/>
-      <c r="C33" s="109"/>
-      <c r="D33" s="110"/>
-      <c r="E33" s="110"/>
-      <c r="F33" s="111"/>
-      <c r="G33" s="95"/>
-      <c r="H33" s="100"/>
-      <c r="I33" s="101"/>
-      <c r="J33" s="101"/>
-      <c r="K33" s="102"/>
+      <c r="B33" s="91"/>
+      <c r="C33" s="87"/>
+      <c r="D33" s="88"/>
+      <c r="E33" s="88"/>
+      <c r="F33" s="89"/>
+      <c r="G33" s="103"/>
+      <c r="H33" s="50"/>
+      <c r="I33" s="51"/>
+      <c r="J33" s="51"/>
+      <c r="K33" s="52"/>
       <c r="L33" s="32"/>
     </row>
     <row r="34" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="92"/>
-      <c r="C34" s="109"/>
-      <c r="D34" s="110"/>
-      <c r="E34" s="110"/>
-      <c r="F34" s="111"/>
-      <c r="G34" s="95"/>
-      <c r="H34" s="100"/>
-      <c r="I34" s="101"/>
-      <c r="J34" s="101"/>
-      <c r="K34" s="102"/>
+      <c r="B34" s="91"/>
+      <c r="C34" s="87"/>
+      <c r="D34" s="88"/>
+      <c r="E34" s="88"/>
+      <c r="F34" s="89"/>
+      <c r="G34" s="103"/>
+      <c r="H34" s="50"/>
+      <c r="I34" s="51"/>
+      <c r="J34" s="51"/>
+      <c r="K34" s="52"/>
       <c r="L34" s="32"/>
     </row>
     <row r="35" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="92"/>
-      <c r="C35" s="109"/>
-      <c r="D35" s="110"/>
-      <c r="E35" s="110"/>
-      <c r="F35" s="111"/>
-      <c r="G35" s="95"/>
-      <c r="H35" s="100"/>
-      <c r="I35" s="101"/>
-      <c r="J35" s="101"/>
-      <c r="K35" s="102"/>
+      <c r="B35" s="91"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="88"/>
+      <c r="E35" s="88"/>
+      <c r="F35" s="89"/>
+      <c r="G35" s="103"/>
+      <c r="H35" s="50"/>
+      <c r="I35" s="51"/>
+      <c r="J35" s="51"/>
+      <c r="K35" s="52"/>
       <c r="L35" s="32"/>
     </row>
     <row r="36" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="92"/>
-      <c r="C36" s="109"/>
-      <c r="D36" s="110"/>
-      <c r="E36" s="110"/>
-      <c r="F36" s="111"/>
-      <c r="G36" s="95"/>
-      <c r="H36" s="100"/>
-      <c r="I36" s="101"/>
-      <c r="J36" s="101"/>
-      <c r="K36" s="102"/>
+      <c r="B36" s="91"/>
+      <c r="C36" s="87"/>
+      <c r="D36" s="88"/>
+      <c r="E36" s="88"/>
+      <c r="F36" s="89"/>
+      <c r="G36" s="103"/>
+      <c r="H36" s="50"/>
+      <c r="I36" s="51"/>
+      <c r="J36" s="51"/>
+      <c r="K36" s="52"/>
       <c r="L36" s="32"/>
     </row>
     <row r="37" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="92"/>
-      <c r="C37" s="109"/>
-      <c r="D37" s="110"/>
-      <c r="E37" s="110"/>
-      <c r="F37" s="111"/>
-      <c r="G37" s="95"/>
-      <c r="H37" s="100"/>
-      <c r="I37" s="101"/>
-      <c r="J37" s="101"/>
-      <c r="K37" s="102"/>
+      <c r="B37" s="91"/>
+      <c r="C37" s="87"/>
+      <c r="D37" s="88"/>
+      <c r="E37" s="88"/>
+      <c r="F37" s="89"/>
+      <c r="G37" s="103"/>
+      <c r="H37" s="50"/>
+      <c r="I37" s="51"/>
+      <c r="J37" s="51"/>
+      <c r="K37" s="52"/>
       <c r="L37" s="32"/>
     </row>
     <row r="38" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="92"/>
-      <c r="C38" s="109"/>
-      <c r="D38" s="110"/>
-      <c r="E38" s="110"/>
-      <c r="F38" s="111"/>
-      <c r="G38" s="95"/>
-      <c r="H38" s="100"/>
-      <c r="I38" s="101"/>
-      <c r="J38" s="101"/>
-      <c r="K38" s="102"/>
+      <c r="B38" s="91"/>
+      <c r="C38" s="87"/>
+      <c r="D38" s="88"/>
+      <c r="E38" s="88"/>
+      <c r="F38" s="89"/>
+      <c r="G38" s="103"/>
+      <c r="H38" s="50"/>
+      <c r="I38" s="51"/>
+      <c r="J38" s="51"/>
+      <c r="K38" s="52"/>
       <c r="L38" s="32"/>
     </row>
     <row r="39" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="92"/>
-      <c r="C39" s="109"/>
-      <c r="D39" s="110"/>
-      <c r="E39" s="110"/>
-      <c r="F39" s="111"/>
-      <c r="G39" s="95"/>
-      <c r="H39" s="100"/>
-      <c r="I39" s="101"/>
-      <c r="J39" s="101"/>
-      <c r="K39" s="102"/>
+      <c r="B39" s="91"/>
+      <c r="C39" s="87"/>
+      <c r="D39" s="88"/>
+      <c r="E39" s="88"/>
+      <c r="F39" s="89"/>
+      <c r="G39" s="103"/>
+      <c r="H39" s="50"/>
+      <c r="I39" s="51"/>
+      <c r="J39" s="51"/>
+      <c r="K39" s="52"/>
       <c r="L39" s="33"/>
     </row>
     <row r="40" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="92"/>
-      <c r="C40" s="109"/>
-      <c r="D40" s="110"/>
-      <c r="E40" s="110"/>
-      <c r="F40" s="111"/>
-      <c r="G40" s="95"/>
-      <c r="H40" s="100"/>
-      <c r="I40" s="101"/>
-      <c r="J40" s="101"/>
-      <c r="K40" s="102"/>
+      <c r="B40" s="91"/>
+      <c r="C40" s="87"/>
+      <c r="D40" s="88"/>
+      <c r="E40" s="88"/>
+      <c r="F40" s="89"/>
+      <c r="G40" s="103"/>
+      <c r="H40" s="50"/>
+      <c r="I40" s="51"/>
+      <c r="J40" s="51"/>
+      <c r="K40" s="52"/>
       <c r="L40" s="33"/>
     </row>
     <row r="41" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="92"/>
-      <c r="C41" s="109"/>
-      <c r="D41" s="110"/>
-      <c r="E41" s="110"/>
-      <c r="F41" s="111"/>
-      <c r="G41" s="95"/>
-      <c r="H41" s="100"/>
-      <c r="I41" s="101"/>
-      <c r="J41" s="101"/>
-      <c r="K41" s="102"/>
+      <c r="B41" s="91"/>
+      <c r="C41" s="87"/>
+      <c r="D41" s="88"/>
+      <c r="E41" s="88"/>
+      <c r="F41" s="89"/>
+      <c r="G41" s="103"/>
+      <c r="H41" s="50"/>
+      <c r="I41" s="51"/>
+      <c r="J41" s="51"/>
+      <c r="K41" s="52"/>
       <c r="L41" s="33"/>
     </row>
     <row r="42" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="92"/>
-      <c r="C42" s="109"/>
-      <c r="D42" s="110"/>
-      <c r="E42" s="110"/>
-      <c r="F42" s="111"/>
-      <c r="G42" s="95"/>
-      <c r="H42" s="100"/>
-      <c r="I42" s="101"/>
-      <c r="J42" s="101"/>
-      <c r="K42" s="102"/>
+      <c r="B42" s="91"/>
+      <c r="C42" s="87"/>
+      <c r="D42" s="88"/>
+      <c r="E42" s="88"/>
+      <c r="F42" s="89"/>
+      <c r="G42" s="103"/>
+      <c r="H42" s="50"/>
+      <c r="I42" s="51"/>
+      <c r="J42" s="51"/>
+      <c r="K42" s="52"/>
       <c r="L42" s="33"/>
     </row>
     <row r="43" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="92"/>
-      <c r="C43" s="109"/>
-      <c r="D43" s="110"/>
-      <c r="E43" s="110"/>
-      <c r="F43" s="111"/>
-      <c r="G43" s="95"/>
-      <c r="H43" s="100"/>
-      <c r="I43" s="101"/>
-      <c r="J43" s="101"/>
-      <c r="K43" s="102"/>
+      <c r="B43" s="91"/>
+      <c r="C43" s="87"/>
+      <c r="D43" s="88"/>
+      <c r="E43" s="88"/>
+      <c r="F43" s="89"/>
+      <c r="G43" s="103"/>
+      <c r="H43" s="50"/>
+      <c r="I43" s="51"/>
+      <c r="J43" s="51"/>
+      <c r="K43" s="52"/>
       <c r="L43" s="33"/>
     </row>
     <row r="44" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="92"/>
-      <c r="C44" s="109"/>
-      <c r="D44" s="110"/>
-      <c r="E44" s="110"/>
-      <c r="F44" s="111"/>
-      <c r="G44" s="95"/>
-      <c r="H44" s="100"/>
-      <c r="I44" s="101"/>
-      <c r="J44" s="101"/>
-      <c r="K44" s="102"/>
+      <c r="B44" s="91"/>
+      <c r="C44" s="87"/>
+      <c r="D44" s="88"/>
+      <c r="E44" s="88"/>
+      <c r="F44" s="89"/>
+      <c r="G44" s="103"/>
+      <c r="H44" s="50"/>
+      <c r="I44" s="51"/>
+      <c r="J44" s="51"/>
+      <c r="K44" s="52"/>
       <c r="L44" s="32"/>
     </row>
     <row r="45" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="92"/>
-      <c r="C45" s="109"/>
-      <c r="D45" s="110"/>
-      <c r="E45" s="110"/>
-      <c r="F45" s="111"/>
-      <c r="G45" s="95"/>
-      <c r="H45" s="100"/>
-      <c r="I45" s="101"/>
-      <c r="J45" s="101"/>
-      <c r="K45" s="102"/>
+      <c r="B45" s="91"/>
+      <c r="C45" s="87"/>
+      <c r="D45" s="88"/>
+      <c r="E45" s="88"/>
+      <c r="F45" s="89"/>
+      <c r="G45" s="103"/>
+      <c r="H45" s="50"/>
+      <c r="I45" s="51"/>
+      <c r="J45" s="51"/>
+      <c r="K45" s="52"/>
       <c r="L45" s="32"/>
     </row>
     <row r="46" spans="2:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="92"/>
-      <c r="C46" s="109"/>
-      <c r="D46" s="110"/>
-      <c r="E46" s="110"/>
-      <c r="F46" s="111"/>
-      <c r="G46" s="95"/>
-      <c r="H46" s="100"/>
-      <c r="I46" s="101"/>
-      <c r="J46" s="101"/>
-      <c r="K46" s="102"/>
+      <c r="B46" s="91"/>
+      <c r="C46" s="87"/>
+      <c r="D46" s="88"/>
+      <c r="E46" s="88"/>
+      <c r="F46" s="89"/>
+      <c r="G46" s="103"/>
+      <c r="H46" s="50"/>
+      <c r="I46" s="51"/>
+      <c r="J46" s="51"/>
+      <c r="K46" s="52"/>
       <c r="L46" s="33"/>
     </row>
     <row r="47" spans="2:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="92"/>
-      <c r="C47" s="109"/>
-      <c r="D47" s="110"/>
-      <c r="E47" s="110"/>
-      <c r="F47" s="111"/>
-      <c r="G47" s="95"/>
-      <c r="H47" s="100"/>
-      <c r="I47" s="101"/>
-      <c r="J47" s="101"/>
-      <c r="K47" s="102"/>
+      <c r="B47" s="91"/>
+      <c r="C47" s="87"/>
+      <c r="D47" s="88"/>
+      <c r="E47" s="88"/>
+      <c r="F47" s="89"/>
+      <c r="G47" s="103"/>
+      <c r="H47" s="50"/>
+      <c r="I47" s="51"/>
+      <c r="J47" s="51"/>
+      <c r="K47" s="52"/>
       <c r="L47" s="33"/>
     </row>
     <row r="48" spans="2:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="92"/>
-      <c r="C48" s="109"/>
-      <c r="D48" s="110"/>
-      <c r="E48" s="110"/>
-      <c r="F48" s="111"/>
-      <c r="G48" s="95"/>
-      <c r="H48" s="100"/>
-      <c r="I48" s="101"/>
-      <c r="J48" s="101"/>
-      <c r="K48" s="102"/>
+      <c r="B48" s="91"/>
+      <c r="C48" s="87"/>
+      <c r="D48" s="88"/>
+      <c r="E48" s="88"/>
+      <c r="F48" s="89"/>
+      <c r="G48" s="103"/>
+      <c r="H48" s="50"/>
+      <c r="I48" s="51"/>
+      <c r="J48" s="51"/>
+      <c r="K48" s="52"/>
       <c r="L48" s="33"/>
     </row>
     <row r="49" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="93"/>
-      <c r="C49" s="112"/>
-      <c r="D49" s="113"/>
-      <c r="E49" s="113"/>
-      <c r="F49" s="114"/>
-      <c r="G49" s="96"/>
-      <c r="H49" s="100"/>
-      <c r="I49" s="101"/>
-      <c r="J49" s="101"/>
-      <c r="K49" s="102"/>
+      <c r="B49" s="92"/>
+      <c r="C49" s="99"/>
+      <c r="D49" s="100"/>
+      <c r="E49" s="100"/>
+      <c r="F49" s="101"/>
+      <c r="G49" s="104"/>
+      <c r="H49" s="50"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="51"/>
+      <c r="K49" s="52"/>
       <c r="L49" s="33"/>
     </row>
     <row r="50" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="92" t="s">
+      <c r="B50" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="C50" s="106"/>
-      <c r="D50" s="107"/>
-      <c r="E50" s="107"/>
-      <c r="F50" s="108"/>
-      <c r="G50" s="103"/>
-      <c r="H50" s="100"/>
-      <c r="I50" s="101"/>
-      <c r="J50" s="101"/>
-      <c r="K50" s="102"/>
+      <c r="C50" s="84"/>
+      <c r="D50" s="85"/>
+      <c r="E50" s="85"/>
+      <c r="F50" s="86"/>
+      <c r="G50" s="93"/>
+      <c r="H50" s="50"/>
+      <c r="I50" s="51"/>
+      <c r="J50" s="51"/>
+      <c r="K50" s="52"/>
       <c r="L50" s="33"/>
     </row>
     <row r="51" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="92"/>
-      <c r="C51" s="109"/>
-      <c r="D51" s="110"/>
-      <c r="E51" s="110"/>
-      <c r="F51" s="111"/>
-      <c r="G51" s="104"/>
-      <c r="H51" s="100"/>
-      <c r="I51" s="101"/>
-      <c r="J51" s="101"/>
-      <c r="K51" s="102"/>
+      <c r="B51" s="91"/>
+      <c r="C51" s="87"/>
+      <c r="D51" s="88"/>
+      <c r="E51" s="88"/>
+      <c r="F51" s="89"/>
+      <c r="G51" s="94"/>
+      <c r="H51" s="50"/>
+      <c r="I51" s="51"/>
+      <c r="J51" s="51"/>
+      <c r="K51" s="52"/>
       <c r="L51" s="33"/>
     </row>
     <row r="52" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="92"/>
-      <c r="C52" s="109"/>
-      <c r="D52" s="110"/>
-      <c r="E52" s="110"/>
-      <c r="F52" s="111"/>
-      <c r="G52" s="104"/>
-      <c r="H52" s="100"/>
-      <c r="I52" s="101"/>
-      <c r="J52" s="101"/>
-      <c r="K52" s="102"/>
+      <c r="B52" s="91"/>
+      <c r="C52" s="87"/>
+      <c r="D52" s="88"/>
+      <c r="E52" s="88"/>
+      <c r="F52" s="89"/>
+      <c r="G52" s="94"/>
+      <c r="H52" s="50"/>
+      <c r="I52" s="51"/>
+      <c r="J52" s="51"/>
+      <c r="K52" s="52"/>
       <c r="L52" s="33"/>
     </row>
     <row r="53" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="92"/>
-      <c r="C53" s="109"/>
-      <c r="D53" s="110"/>
-      <c r="E53" s="110"/>
-      <c r="F53" s="111"/>
-      <c r="G53" s="104"/>
-      <c r="H53" s="100"/>
-      <c r="I53" s="101"/>
-      <c r="J53" s="101"/>
-      <c r="K53" s="102"/>
+      <c r="B53" s="91"/>
+      <c r="C53" s="87"/>
+      <c r="D53" s="88"/>
+      <c r="E53" s="88"/>
+      <c r="F53" s="89"/>
+      <c r="G53" s="94"/>
+      <c r="H53" s="50"/>
+      <c r="I53" s="51"/>
+      <c r="J53" s="51"/>
+      <c r="K53" s="52"/>
       <c r="L53" s="33"/>
     </row>
     <row r="54" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="92"/>
-      <c r="C54" s="109"/>
-      <c r="D54" s="110"/>
-      <c r="E54" s="110"/>
-      <c r="F54" s="111"/>
-      <c r="G54" s="104"/>
-      <c r="H54" s="100"/>
-      <c r="I54" s="101"/>
-      <c r="J54" s="101"/>
-      <c r="K54" s="102"/>
+      <c r="B54" s="91"/>
+      <c r="C54" s="87"/>
+      <c r="D54" s="88"/>
+      <c r="E54" s="88"/>
+      <c r="F54" s="89"/>
+      <c r="G54" s="94"/>
+      <c r="H54" s="50"/>
+      <c r="I54" s="51"/>
+      <c r="J54" s="51"/>
+      <c r="K54" s="52"/>
       <c r="L54" s="33"/>
     </row>
     <row r="55" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="92"/>
-      <c r="C55" s="109"/>
-      <c r="D55" s="110"/>
-      <c r="E55" s="110"/>
-      <c r="F55" s="111"/>
-      <c r="G55" s="104"/>
-      <c r="H55" s="100"/>
-      <c r="I55" s="101"/>
-      <c r="J55" s="101"/>
-      <c r="K55" s="102"/>
+      <c r="B55" s="91"/>
+      <c r="C55" s="87"/>
+      <c r="D55" s="88"/>
+      <c r="E55" s="88"/>
+      <c r="F55" s="89"/>
+      <c r="G55" s="94"/>
+      <c r="H55" s="50"/>
+      <c r="I55" s="51"/>
+      <c r="J55" s="51"/>
+      <c r="K55" s="52"/>
       <c r="L55" s="33"/>
     </row>
     <row r="56" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="92"/>
-      <c r="C56" s="109"/>
-      <c r="D56" s="110"/>
-      <c r="E56" s="110"/>
-      <c r="F56" s="111"/>
-      <c r="G56" s="104"/>
-      <c r="H56" s="100"/>
-      <c r="I56" s="101"/>
-      <c r="J56" s="101"/>
-      <c r="K56" s="102"/>
+      <c r="B56" s="91"/>
+      <c r="C56" s="87"/>
+      <c r="D56" s="88"/>
+      <c r="E56" s="88"/>
+      <c r="F56" s="89"/>
+      <c r="G56" s="94"/>
+      <c r="H56" s="50"/>
+      <c r="I56" s="51"/>
+      <c r="J56" s="51"/>
+      <c r="K56" s="52"/>
       <c r="L56" s="33"/>
     </row>
     <row r="57" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="92"/>
-      <c r="C57" s="109"/>
-      <c r="D57" s="110"/>
-      <c r="E57" s="110"/>
-      <c r="F57" s="111"/>
-      <c r="G57" s="104"/>
-      <c r="H57" s="100"/>
-      <c r="I57" s="101"/>
-      <c r="J57" s="101"/>
-      <c r="K57" s="102"/>
+      <c r="B57" s="91"/>
+      <c r="C57" s="87"/>
+      <c r="D57" s="88"/>
+      <c r="E57" s="88"/>
+      <c r="F57" s="89"/>
+      <c r="G57" s="94"/>
+      <c r="H57" s="50"/>
+      <c r="I57" s="51"/>
+      <c r="J57" s="51"/>
+      <c r="K57" s="52"/>
       <c r="L57" s="33"/>
     </row>
     <row r="58" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="92"/>
-      <c r="C58" s="109"/>
-      <c r="D58" s="110"/>
-      <c r="E58" s="110"/>
-      <c r="F58" s="111"/>
-      <c r="G58" s="104"/>
-      <c r="H58" s="100"/>
-      <c r="I58" s="101"/>
-      <c r="J58" s="101"/>
-      <c r="K58" s="102"/>
+      <c r="B58" s="91"/>
+      <c r="C58" s="87"/>
+      <c r="D58" s="88"/>
+      <c r="E58" s="88"/>
+      <c r="F58" s="89"/>
+      <c r="G58" s="94"/>
+      <c r="H58" s="50"/>
+      <c r="I58" s="51"/>
+      <c r="J58" s="51"/>
+      <c r="K58" s="52"/>
       <c r="L58" s="33"/>
     </row>
     <row r="59" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="92"/>
-      <c r="C59" s="109"/>
-      <c r="D59" s="110"/>
-      <c r="E59" s="110"/>
-      <c r="F59" s="111"/>
-      <c r="G59" s="104"/>
-      <c r="H59" s="100"/>
-      <c r="I59" s="101"/>
-      <c r="J59" s="101"/>
-      <c r="K59" s="102"/>
+      <c r="B59" s="91"/>
+      <c r="C59" s="87"/>
+      <c r="D59" s="88"/>
+      <c r="E59" s="88"/>
+      <c r="F59" s="89"/>
+      <c r="G59" s="94"/>
+      <c r="H59" s="50"/>
+      <c r="I59" s="51"/>
+      <c r="J59" s="51"/>
+      <c r="K59" s="52"/>
       <c r="L59" s="33"/>
     </row>
     <row r="60" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="92"/>
-      <c r="C60" s="109"/>
-      <c r="D60" s="110"/>
-      <c r="E60" s="110"/>
-      <c r="F60" s="111"/>
-      <c r="G60" s="104"/>
-      <c r="H60" s="100"/>
-      <c r="I60" s="101"/>
-      <c r="J60" s="101"/>
-      <c r="K60" s="102"/>
+      <c r="B60" s="91"/>
+      <c r="C60" s="87"/>
+      <c r="D60" s="88"/>
+      <c r="E60" s="88"/>
+      <c r="F60" s="89"/>
+      <c r="G60" s="94"/>
+      <c r="H60" s="50"/>
+      <c r="I60" s="51"/>
+      <c r="J60" s="51"/>
+      <c r="K60" s="52"/>
       <c r="L60" s="33"/>
     </row>
     <row r="61" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="93"/>
-      <c r="C61" s="109"/>
-      <c r="D61" s="110"/>
-      <c r="E61" s="110"/>
-      <c r="F61" s="111"/>
-      <c r="G61" s="105"/>
-      <c r="H61" s="100"/>
-      <c r="I61" s="101"/>
-      <c r="J61" s="101"/>
-      <c r="K61" s="102"/>
+      <c r="B61" s="92"/>
+      <c r="C61" s="87"/>
+      <c r="D61" s="88"/>
+      <c r="E61" s="88"/>
+      <c r="F61" s="89"/>
+      <c r="G61" s="95"/>
+      <c r="H61" s="50"/>
+      <c r="I61" s="51"/>
+      <c r="J61" s="51"/>
+      <c r="K61" s="52"/>
       <c r="L61" s="33"/>
     </row>
     <row r="62" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="91" t="s">
+      <c r="B62" s="90" t="s">
         <v>15</v>
       </c>
-      <c r="C62" s="106"/>
-      <c r="D62" s="107"/>
-      <c r="E62" s="107"/>
-      <c r="F62" s="108"/>
-      <c r="G62" s="103"/>
-      <c r="H62" s="100"/>
-      <c r="I62" s="101"/>
-      <c r="J62" s="101"/>
-      <c r="K62" s="102"/>
+      <c r="C62" s="84"/>
+      <c r="D62" s="85"/>
+      <c r="E62" s="85"/>
+      <c r="F62" s="86"/>
+      <c r="G62" s="93"/>
+      <c r="H62" s="50"/>
+      <c r="I62" s="51"/>
+      <c r="J62" s="51"/>
+      <c r="K62" s="52"/>
       <c r="L62" s="33"/>
     </row>
     <row r="63" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="92"/>
-      <c r="C63" s="109"/>
-      <c r="D63" s="110"/>
-      <c r="E63" s="110"/>
-      <c r="F63" s="111"/>
-      <c r="G63" s="104"/>
-      <c r="H63" s="100"/>
-      <c r="I63" s="101"/>
-      <c r="J63" s="101"/>
-      <c r="K63" s="102"/>
+      <c r="B63" s="91"/>
+      <c r="C63" s="87"/>
+      <c r="D63" s="88"/>
+      <c r="E63" s="88"/>
+      <c r="F63" s="89"/>
+      <c r="G63" s="94"/>
+      <c r="H63" s="50"/>
+      <c r="I63" s="51"/>
+      <c r="J63" s="51"/>
+      <c r="K63" s="52"/>
       <c r="L63" s="33"/>
     </row>
     <row r="64" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="92"/>
-      <c r="C64" s="109"/>
-      <c r="D64" s="110"/>
-      <c r="E64" s="110"/>
-      <c r="F64" s="111"/>
-      <c r="G64" s="104"/>
-      <c r="H64" s="100"/>
-      <c r="I64" s="101"/>
-      <c r="J64" s="101"/>
-      <c r="K64" s="102"/>
+      <c r="B64" s="91"/>
+      <c r="C64" s="87"/>
+      <c r="D64" s="88"/>
+      <c r="E64" s="88"/>
+      <c r="F64" s="89"/>
+      <c r="G64" s="94"/>
+      <c r="H64" s="50"/>
+      <c r="I64" s="51"/>
+      <c r="J64" s="51"/>
+      <c r="K64" s="52"/>
       <c r="L64" s="33"/>
     </row>
     <row r="65" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="92"/>
-      <c r="C65" s="109"/>
-      <c r="D65" s="110"/>
-      <c r="E65" s="110"/>
-      <c r="F65" s="111"/>
-      <c r="G65" s="104"/>
-      <c r="H65" s="100"/>
-      <c r="I65" s="101"/>
-      <c r="J65" s="101"/>
-      <c r="K65" s="102"/>
+      <c r="B65" s="91"/>
+      <c r="C65" s="87"/>
+      <c r="D65" s="88"/>
+      <c r="E65" s="88"/>
+      <c r="F65" s="89"/>
+      <c r="G65" s="94"/>
+      <c r="H65" s="50"/>
+      <c r="I65" s="51"/>
+      <c r="J65" s="51"/>
+      <c r="K65" s="52"/>
       <c r="L65" s="33"/>
     </row>
     <row r="66" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="92"/>
-      <c r="C66" s="109"/>
-      <c r="D66" s="110"/>
-      <c r="E66" s="110"/>
-      <c r="F66" s="111"/>
-      <c r="G66" s="104"/>
-      <c r="H66" s="100"/>
-      <c r="I66" s="101"/>
-      <c r="J66" s="101"/>
-      <c r="K66" s="102"/>
+      <c r="B66" s="91"/>
+      <c r="C66" s="87"/>
+      <c r="D66" s="88"/>
+      <c r="E66" s="88"/>
+      <c r="F66" s="89"/>
+      <c r="G66" s="94"/>
+      <c r="H66" s="50"/>
+      <c r="I66" s="51"/>
+      <c r="J66" s="51"/>
+      <c r="K66" s="52"/>
       <c r="L66" s="33"/>
     </row>
     <row r="67" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="92"/>
-      <c r="C67" s="109"/>
-      <c r="D67" s="110"/>
-      <c r="E67" s="110"/>
-      <c r="F67" s="111"/>
-      <c r="G67" s="104"/>
-      <c r="H67" s="100"/>
-      <c r="I67" s="101"/>
-      <c r="J67" s="101"/>
-      <c r="K67" s="102"/>
+      <c r="B67" s="91"/>
+      <c r="C67" s="87"/>
+      <c r="D67" s="88"/>
+      <c r="E67" s="88"/>
+      <c r="F67" s="89"/>
+      <c r="G67" s="94"/>
+      <c r="H67" s="50"/>
+      <c r="I67" s="51"/>
+      <c r="J67" s="51"/>
+      <c r="K67" s="52"/>
     </row>
     <row r="68" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="93"/>
-      <c r="C68" s="109"/>
-      <c r="D68" s="110"/>
-      <c r="E68" s="110"/>
-      <c r="F68" s="111"/>
-      <c r="G68" s="105"/>
-      <c r="H68" s="115"/>
-      <c r="I68" s="116"/>
-      <c r="J68" s="116"/>
-      <c r="K68" s="117"/>
+      <c r="B68" s="92"/>
+      <c r="C68" s="87"/>
+      <c r="D68" s="88"/>
+      <c r="E68" s="88"/>
+      <c r="F68" s="89"/>
+      <c r="G68" s="95"/>
+      <c r="H68" s="96"/>
+      <c r="I68" s="97"/>
+      <c r="J68" s="97"/>
+      <c r="K68" s="98"/>
     </row>
     <row r="69" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B69" s="1"/>
-      <c r="C69" s="118" t="s">
+      <c r="C69" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="D69" s="119"/>
-      <c r="E69" s="120"/>
+      <c r="D69" s="57"/>
+      <c r="E69" s="58"/>
       <c r="F69" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="G69" s="121"/>
-      <c r="H69" s="122"/>
+      <c r="G69" s="64"/>
+      <c r="H69" s="65"/>
       <c r="I69" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="J69" s="123"/>
-      <c r="K69" s="124"/>
+      <c r="J69" s="66"/>
+      <c r="K69" s="67"/>
     </row>
     <row r="70" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="7"/>
       <c r="C70" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="D70" s="125" t="s">
+      <c r="D70" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="E70" s="126"/>
+      <c r="E70" s="69"/>
       <c r="F70" s="36"/>
       <c r="G70" s="37"/>
       <c r="H70" s="37"/>
@@ -8671,26 +8671,26 @@
     <row r="71" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B71" s="7"/>
       <c r="C71" s="39"/>
-      <c r="D71" s="127"/>
-      <c r="E71" s="128"/>
+      <c r="D71" s="70"/>
+      <c r="E71" s="71"/>
       <c r="F71" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="G71" s="131"/>
-      <c r="H71" s="132"/>
+      <c r="G71" s="74"/>
+      <c r="H71" s="75"/>
       <c r="I71" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="J71" s="129"/>
-      <c r="K71" s="130"/>
+      <c r="J71" s="72"/>
+      <c r="K71" s="73"/>
     </row>
     <row r="72" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B72" s="7"/>
-      <c r="C72" s="118" t="s">
+      <c r="C72" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="D72" s="119"/>
-      <c r="E72" s="120"/>
+      <c r="D72" s="57"/>
+      <c r="E72" s="58"/>
       <c r="F72" s="36"/>
       <c r="G72" s="37"/>
       <c r="H72" s="37"/>
@@ -8703,28 +8703,28 @@
       <c r="C73" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="D73" s="133" t="s">
+      <c r="D73" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="E73" s="134"/>
+      <c r="E73" s="77"/>
       <c r="F73" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="G73" s="135"/>
-      <c r="H73" s="136"/>
+      <c r="G73" s="78"/>
+      <c r="H73" s="79"/>
       <c r="I73" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="J73" s="137" t="s">
+      <c r="J73" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="K73" s="138"/>
+      <c r="K73" s="81"/>
     </row>
     <row r="74" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B74" s="42"/>
       <c r="C74" s="43"/>
-      <c r="D74" s="139"/>
-      <c r="E74" s="140"/>
+      <c r="D74" s="82"/>
+      <c r="E74" s="83"/>
       <c r="F74" s="42"/>
       <c r="G74" s="11"/>
       <c r="H74" s="11"/>
@@ -8734,11 +8734,11 @@
     </row>
     <row r="75" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B75" s="42"/>
-      <c r="C75" s="118" t="s">
+      <c r="C75" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D75" s="119"/>
-      <c r="E75" s="120"/>
+      <c r="D75" s="57"/>
+      <c r="E75" s="58"/>
       <c r="F75" s="42"/>
       <c r="G75" s="11"/>
       <c r="H75" s="11"/>
@@ -8748,9 +8748,9 @@
     </row>
     <row r="76" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B76" s="42"/>
-      <c r="C76" s="141"/>
-      <c r="D76" s="142"/>
-      <c r="E76" s="143"/>
+      <c r="C76" s="53"/>
+      <c r="D76" s="54"/>
+      <c r="E76" s="55"/>
       <c r="F76" s="42"/>
       <c r="G76" s="11"/>
       <c r="H76" s="11"/>
@@ -8760,34 +8760,34 @@
     </row>
     <row r="77" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B77" s="7"/>
-      <c r="C77" s="118" t="s">
+      <c r="C77" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="D77" s="119"/>
-      <c r="E77" s="120"/>
+      <c r="D77" s="57"/>
+      <c r="E77" s="58"/>
       <c r="F77" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="G77" s="144" t="s">
-        <v>30</v>
+      <c r="G77" s="59" t="s">
+        <v>31</v>
       </c>
-      <c r="H77" s="145"/>
+      <c r="H77" s="60"/>
       <c r="I77" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="J77" s="144" t="s">
-        <v>31</v>
+      <c r="J77" s="59" t="s">
+        <v>32</v>
       </c>
-      <c r="K77" s="145"/>
+      <c r="K77" s="60"/>
     </row>
     <row r="78" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B78" s="45"/>
-      <c r="C78" s="146">
+      <c r="C78" s="61">
         <f>(D74-C74)+C71+D71</f>
         <v>0</v>
       </c>
-      <c r="D78" s="147"/>
-      <c r="E78" s="148"/>
+      <c r="D78" s="62"/>
+      <c r="E78" s="63"/>
       <c r="F78" s="46"/>
       <c r="G78" s="47"/>
       <c r="H78" s="48"/>
@@ -8806,6 +8806,85 @@
     </row>
   </sheetData>
   <mergeCells count="103">
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:K7"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="K1:K3"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="D3:G3"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="G14:K14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="G10:K10"/>
+    <mergeCell ref="G11:K11"/>
+    <mergeCell ref="H32:K32"/>
+    <mergeCell ref="H33:K33"/>
+    <mergeCell ref="H40:K40"/>
+    <mergeCell ref="B16:B49"/>
+    <mergeCell ref="G16:G49"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="H28:K28"/>
+    <mergeCell ref="H29:K29"/>
+    <mergeCell ref="H30:K30"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="H27:K27"/>
+    <mergeCell ref="H34:K34"/>
+    <mergeCell ref="H35:K35"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="H22:K22"/>
+    <mergeCell ref="H49:K49"/>
+    <mergeCell ref="B50:B61"/>
+    <mergeCell ref="G50:G61"/>
+    <mergeCell ref="H50:K50"/>
+    <mergeCell ref="H51:K51"/>
+    <mergeCell ref="H52:K52"/>
+    <mergeCell ref="H59:K59"/>
+    <mergeCell ref="H60:K60"/>
+    <mergeCell ref="H61:K61"/>
+    <mergeCell ref="H56:K56"/>
+    <mergeCell ref="C16:F49"/>
+    <mergeCell ref="H41:K41"/>
+    <mergeCell ref="H42:K42"/>
+    <mergeCell ref="H37:K37"/>
+    <mergeCell ref="H38:K38"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H47:K47"/>
+    <mergeCell ref="H48:K48"/>
+    <mergeCell ref="H43:K43"/>
+    <mergeCell ref="H44:K44"/>
+    <mergeCell ref="H45:K45"/>
+    <mergeCell ref="H36:K36"/>
+    <mergeCell ref="H31:K31"/>
+    <mergeCell ref="H53:K53"/>
+    <mergeCell ref="H54:K54"/>
+    <mergeCell ref="H55:K55"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="G62:G68"/>
+    <mergeCell ref="H62:K62"/>
+    <mergeCell ref="H63:K63"/>
+    <mergeCell ref="H64:K64"/>
+    <mergeCell ref="H65:K65"/>
+    <mergeCell ref="H66:K66"/>
+    <mergeCell ref="H67:K67"/>
+    <mergeCell ref="H68:K68"/>
+    <mergeCell ref="C62:F68"/>
     <mergeCell ref="H23:K23"/>
     <mergeCell ref="H24:K24"/>
     <mergeCell ref="H25:K25"/>
@@ -8830,85 +8909,6 @@
     <mergeCell ref="H57:K57"/>
     <mergeCell ref="H58:K58"/>
     <mergeCell ref="C50:F61"/>
-    <mergeCell ref="H53:K53"/>
-    <mergeCell ref="H54:K54"/>
-    <mergeCell ref="H55:K55"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="G62:G68"/>
-    <mergeCell ref="H62:K62"/>
-    <mergeCell ref="H63:K63"/>
-    <mergeCell ref="H64:K64"/>
-    <mergeCell ref="H65:K65"/>
-    <mergeCell ref="H66:K66"/>
-    <mergeCell ref="H67:K67"/>
-    <mergeCell ref="H68:K68"/>
-    <mergeCell ref="C62:F68"/>
-    <mergeCell ref="H49:K49"/>
-    <mergeCell ref="B50:B61"/>
-    <mergeCell ref="G50:G61"/>
-    <mergeCell ref="H50:K50"/>
-    <mergeCell ref="H51:K51"/>
-    <mergeCell ref="H52:K52"/>
-    <mergeCell ref="H59:K59"/>
-    <mergeCell ref="H60:K60"/>
-    <mergeCell ref="H61:K61"/>
-    <mergeCell ref="H56:K56"/>
-    <mergeCell ref="C16:F49"/>
-    <mergeCell ref="H41:K41"/>
-    <mergeCell ref="H42:K42"/>
-    <mergeCell ref="H37:K37"/>
-    <mergeCell ref="H38:K38"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="H46:K46"/>
-    <mergeCell ref="H47:K47"/>
-    <mergeCell ref="H48:K48"/>
-    <mergeCell ref="H43:K43"/>
-    <mergeCell ref="H44:K44"/>
-    <mergeCell ref="H45:K45"/>
-    <mergeCell ref="H36:K36"/>
-    <mergeCell ref="H31:K31"/>
-    <mergeCell ref="H32:K32"/>
-    <mergeCell ref="H33:K33"/>
-    <mergeCell ref="H40:K40"/>
-    <mergeCell ref="B16:B49"/>
-    <mergeCell ref="G16:G49"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="H28:K28"/>
-    <mergeCell ref="H29:K29"/>
-    <mergeCell ref="H30:K30"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="H27:K27"/>
-    <mergeCell ref="H34:K34"/>
-    <mergeCell ref="H35:K35"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="H22:K22"/>
-    <mergeCell ref="G12:K12"/>
-    <mergeCell ref="G13:K13"/>
-    <mergeCell ref="G14:K14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:K9"/>
-    <mergeCell ref="G10:K10"/>
-    <mergeCell ref="G11:K11"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:K7"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="K1:K3"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="D3:G3"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="D4:G4"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="K4:K5"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>